<commit_message>
Update: Chennai-April-2025 by superadmin
</commit_message>
<xml_diff>
--- a/Chennai-April-2025.xlsx
+++ b/Chennai-April-2025.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2023031\Documents\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A5AF7B-DD94-4C1F-9BCB-6A3BA4E14AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -136,23 +142,23 @@
     <t>TN14AK9389</t>
   </si>
   <si>
-    <t>Etios</t>
-  </si>
-  <si>
     <t>CRYSTA</t>
   </si>
   <si>
     <t>CITROEN</t>
+  </si>
+  <si>
+    <t>ETIOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,13 +222,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -260,7 +274,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -294,6 +308,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -328,9 +343,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -503,11 +519,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -590,7 +606,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>47</v>
       </c>
@@ -607,7 +623,7 @@
         <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G2" s="2">
         <v>42979</v>
@@ -670,7 +686,7 @@
         <v>51.94</v>
       </c>
     </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>48</v>
       </c>
@@ -687,7 +703,7 @@
         <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G3" s="2">
         <v>43249</v>
@@ -750,7 +766,7 @@
         <v>57.84</v>
       </c>
     </row>
-    <row r="4" spans="1:27">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>49</v>
       </c>
@@ -767,7 +783,7 @@
         <v>31</v>
       </c>
       <c r="F4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G4" s="2">
         <v>43290</v>
@@ -830,7 +846,7 @@
         <v>52.66</v>
       </c>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>50</v>
       </c>
@@ -847,7 +863,7 @@
         <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G5" s="2">
         <v>44874</v>
@@ -910,7 +926,7 @@
         <v>54.39</v>
       </c>
     </row>
-    <row r="6" spans="1:27">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>51</v>
       </c>
@@ -927,7 +943,7 @@
         <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G6" s="2">
         <v>44874</v>
@@ -990,7 +1006,7 @@
         <v>59.9</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>52</v>
       </c>
@@ -1007,7 +1023,7 @@
         <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G7" s="2">
         <v>44874</v>
@@ -1070,7 +1086,7 @@
         <v>57.45</v>
       </c>
     </row>
-    <row r="8" spans="1:27">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>53</v>
       </c>
@@ -1087,7 +1103,7 @@
         <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G8" s="2">
         <v>43643</v>
@@ -1150,7 +1166,7 @@
         <v>41.97</v>
       </c>
     </row>
-    <row r="9" spans="1:27">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>54</v>
       </c>
@@ -1167,7 +1183,7 @@
         <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G9" s="2">
         <v>43249</v>
@@ -1230,7 +1246,7 @@
         <v>24.58</v>
       </c>
     </row>
-    <row r="10" spans="1:27">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>55</v>
       </c>
@@ -1247,7 +1263,7 @@
         <v>37</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G10" s="2">
         <v>43724</v>
@@ -1310,7 +1326,7 @@
         <v>54.37</v>
       </c>
     </row>
-    <row r="11" spans="1:27">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>56</v>
       </c>
@@ -1327,7 +1343,7 @@
         <v>38</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G11" s="2">
         <v>45348</v>
@@ -1390,7 +1406,7 @@
         <v>13.04</v>
       </c>
     </row>
-    <row r="12" spans="1:27">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>57</v>
       </c>
@@ -1407,7 +1423,7 @@
         <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G12" s="2">
         <v>45502</v>
@@ -1472,5 +1488,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Revvity Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a1b582e8-0077-416f-9765-e019f2ce0792}" enabled="1" method="Standard" siteId="{66a92d0f-8ca8-403c-84e6-5503c5643994}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>